<commit_message>
feat: complete dynamic health audit, profile realtime synchronization, and expo navigation responsiveness
</commit_message>
<xml_diff>
--- a/vitalcore-expo/Test Results/Excel/Execution_Summary.xlsx
+++ b/vitalcore-expo/Test Results/Excel/Execution_Summary.xlsx
@@ -22,7 +22,7 @@
     <t>Generated At</t>
   </si>
   <si>
-    <t>21/8/2026, 10:16:10 pm</t>
+    <t>22/8/2026, 12:07:39 am</t>
   </si>
   <si>
     <t>Platform</t>
@@ -474,7 +474,7 @@
         <v>6</v>
       </c>
       <c r="B4" s="2">
-        <v>30</v>
+        <v>300</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -482,7 +482,7 @@
         <v>7</v>
       </c>
       <c r="B5" s="2">
-        <v>30</v>
+        <v>300</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>